<commit_message>
paper run 2026-08-29 02:06
</commit_message>
<xml_diff>
--- a/reports/2026-08-28.xlsx
+++ b/reports/2026-08-28.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сделки" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итоги" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Сделки" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Итоги" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -859,6 +859,350 @@
       </c>
       <c r="K10" t="n">
         <v>4.06</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-28T13:58:48.997714+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F11" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="G11" t="n">
+        <v>12.23</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-0.00084</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>5.75</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28T14:28:46.183771+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="G12" t="n">
+        <v>13.67</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-0.00159</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>-7.52</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-28T14:28:46.646557+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="G13" t="n">
+        <v>13.58</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-0.00122</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>-7.33</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-28T16:11:20.120355+00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="G14" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.757</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>-5.45</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-28T16:56:29.547414+00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="G15" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>2.15</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-28T17:08:54.324475+00:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F16" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="G16" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.00086</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>6.02</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-28T17:43:58.102127+00:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.00087</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>2.88</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-28T21:41:16.633819+00:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6.76</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.776</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-0.00168</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>2.71</v>
       </c>
     </row>
   </sheetData>
@@ -872,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -894,7 +1238,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -904,7 +1248,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -914,7 +1258,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -924,7 +1268,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.5882352941176471</v>
       </c>
     </row>
     <row r="6">
@@ -934,7 +1278,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-7.11</v>
+        <v>-7.9</v>
       </c>
     </row>
     <row r="7">
@@ -944,7 +1288,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20.46</v>
+        <v>39.97</v>
       </c>
     </row>
     <row r="8">
@@ -954,7 +1298,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-27.57</v>
+        <v>-47.87</v>
       </c>
     </row>
     <row r="9">
@@ -964,7 +1308,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.74</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="10">
@@ -974,287 +1318,744 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>92.89000000000001</v>
+        <v>92.10000000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
+          <t>QUALIFYING SIGNALS (hypothetical — не реальные деньги)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>7</v>
-      </c>
-      <c r="C13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" t="n">
-        <v>-13.45</v>
+          <t>Срез</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>сигналов</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>hypothetical P&amp;L</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>realized P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+          <t>По окнам</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
         <v>2</v>
       </c>
-      <c r="C14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" t="n">
-        <v>6.34</v>
+      <c r="D15" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.71</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
+          <t>По активам</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>-1.39</v>
+        <v>-1.53</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.71</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>-5.72</v>
+        <v>3.71</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>00</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.28</v>
+        <v>2.71</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.71</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>2</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
-        <v>-14.87</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>1</v>
       </c>
       <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="E23" t="n">
         <v>0</v>
-      </c>
-      <c r="D23" t="n">
-        <v>-6.63</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>NO_LIQUIDITY</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>6.34</v>
+        <v>-4.24</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>8.33</v>
+        <v>2.71</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2.71</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>0.50</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>4</v>
-      </c>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" t="n">
-        <v>-15.71</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0.55</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" t="n">
-        <v>4.27</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>-7.33</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-7.52</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-2.57</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="n">
+        <v>9.52</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>8</v>
+      </c>
+      <c r="C36" t="n">
+        <v>5</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-1.98</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>9</v>
+      </c>
+      <c r="C37" t="n">
+        <v>5</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-5.92</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-0.28</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>-14.87</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>-6.63</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>6.34</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="n">
+        <v>8.33</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>5.75</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-14.85</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-3.3</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>2.71</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>8</v>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="n">
+        <v>-8.390000000000001</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-8.699999999999999</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2.71</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>0.60</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B55" t="n">
+        <v>5</v>
+      </c>
+      <c r="C55" t="n">
         <v>4</v>
       </c>
-      <c r="C30" t="n">
-        <v>3</v>
-      </c>
-      <c r="D30" t="n">
-        <v>4.33</v>
+      <c r="D55" t="n">
+        <v>6.48</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>2.71</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>16</v>
+      </c>
+      <c r="C59" t="n">
+        <v>9</v>
+      </c>
+      <c r="D59" t="n">
+        <v>-10.61</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>8</v>
+      </c>
+      <c r="C62" t="n">
+        <v>6</v>
+      </c>
+      <c r="D62" t="n">
+        <v>10.71</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>9</v>
+      </c>
+      <c r="C63" t="n">
+        <v>4</v>
+      </c>
+      <c r="D63" t="n">
+        <v>-18.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>